<commit_message>
Geboortedatum beslist: 01/01/1900 voor iedereen
Novel maakt naam en geboortedatum verplicht omdat de software voor klinische
dossiers gebouwd is. De PI beslist vandaag dat daar een vaste dummydatum in
gaat, voor elke deelnemer dezelfde, naast de X in beide naamvelden.

Een gevolg dat het vermelden waard is: het veld Age in Visits wordt uit de
geboortedatum berekend en komt daarmee op 126 uit. Dat is geen fout maar het
zichtbare teken dat er geen echte geboortedatum in staat -- wie de database
opent, ziet meteen dat dit een plaatshouder is en niet per ongeluk een leeg
gelaten veld. De werkelijke leeftijd staat in de eCRF. Dat staat er nu bij,
zodat niemand het later gaat 'verbeteren'.

Het openstaande punt hierover vervalt in de SOP, in de tijdlijn en in de
afvinklijst.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARADISE_WP1_afvinklijst.xlsx
+++ b/PARADISE_WP1_afvinklijst.xlsx
@@ -4279,9 +4279,9 @@
   <autoFilter ref="A4:I79"/>
   <mergeCells count="11">
     <mergeCell ref="A65:I65"/>
-    <mergeCell ref="A41:I41"/>
     <mergeCell ref="A73:I73"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A41:I41"/>
     <mergeCell ref="A5:I5"/>
     <mergeCell ref="A60:I60"/>
     <mergeCell ref="A1:I1"/>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="C47" s="23" t="inlineStr">
         <is>
-          <t>Novel vraagt een geboortedatum in het veld Persons. Samen met een centrum en een meetdatum is dat herleidbaar. Beslissen: alleen het geboortejaar, of het veld leeg laten.</t>
+          <t>Beslist: 01/01/1900 voor elke deelnemer, samen met een X in beide naamvelden. Het afgeleide veld Age komt daardoor op 126 — dat maakt meteen zichtbaar dat het een plaatshouder is. De werkelijke leeftijd staat in de eCRF.</t>
         </is>
       </c>
       <c r="D47" s="23" t="inlineStr">
@@ -5650,17 +5650,17 @@
       </c>
       <c r="E47" s="23" t="inlineStr">
         <is>
-          <t>Hoog</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F47" s="23" t="inlineStr">
         <is>
-          <t>Te doen</t>
+          <t>Klaar</t>
         </is>
       </c>
       <c r="G47" s="23" t="inlineStr">
         <is>
-          <t>GDPR — vastgesteld 14 sep</t>
+          <t>Beslissing PI 14 sep</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Vier regels in de afvinklijst bijgewerkt naar wat er al gedaan is
De lijst zei nog dat de werkinstructie pedar volledig ontbreekt en dat er nog
een veld voor de schermafbeelding moet komen. Allebei bestaan ze. Ook de
identificatie in Persons en de route van de meetbestanden staan nu op wat er
werkelijk beslist is, met erbij wat er nog rest: het datamanagementplan, en
de weg van het geexporteerde pedar-bestand zelf.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARADISE_WP1_afvinklijst.xlsx
+++ b/PARADISE_WP1_afvinklijst.xlsx
@@ -4279,9 +4279,9 @@
   <autoFilter ref="A4:I79"/>
   <mergeCells count="11">
     <mergeCell ref="A65:I65"/>
-    <mergeCell ref="A41:I41"/>
     <mergeCell ref="A73:I73"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A41:I41"/>
     <mergeCell ref="A5:I5"/>
     <mergeCell ref="A60:I60"/>
     <mergeCell ref="A1:I1"/>
@@ -4349,7 +4349,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="26.1" customHeight="1" s="14">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -4781,7 +4780,7 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Ontbreekt volledig; voor MoveMonitor (19b) en Orthotimer (25b) bestaat er wel een</t>
+          <t>Gedaan: eCRF 09b bestaat, 18 hoofdstukken, 55 stappen, 17 figuren. Nog 7 openstaande punten achteraan het document.</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -4796,12 +4795,12 @@
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>Te doen</t>
+          <t>Klaar</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>Toestel waarop de klinische beslissing rust</t>
+          <t>Afgewerkt 14 sep</t>
         </is>
       </c>
     </row>
@@ -4996,7 +4995,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
@@ -5211,7 +5209,7 @@
       </c>
       <c r="C34" s="23" t="inlineStr">
         <is>
-          <t>Per deelnemer, meetmoment en conditie een plek om het MPP-beeld in te plakken, plus velden voor de drie hoogste waarden met hun plaats</t>
+          <t>Gedaan: het blad 'Meting' van de Pressure Monitoring Tool heeft blok 4 voor de drie hoogste waarden met hun plaats en blok 6 voor de twee schermafbeeldingen, per conditie.</t>
         </is>
       </c>
       <c r="D34" s="23" t="inlineStr">
@@ -5226,12 +5224,12 @@
       </c>
       <c r="F34" s="23" t="inlineStr">
         <is>
-          <t>Te doen</t>
+          <t>Klaar</t>
         </is>
       </c>
       <c r="G34" s="23" t="inlineStr">
         <is>
-          <t>Volgt uit de beslissing van 11 sep</t>
+          <t>Afgewerkt 14 sep</t>
         </is>
       </c>
     </row>
@@ -5409,7 +5407,7 @@
       </c>
       <c r="C40" s="23" t="inlineStr">
         <is>
-          <t>De database vraagt uit zichzelf naam en geboortedatum. Vastleggen dat er uitsluitend de deelnemerscode in gaat, en dat in de SOP en het datamanagementplan zetten.</t>
+          <t>Beslist en in de SOP verwerkt: deelnemerscode in ID en External ID, X in beide naamvelden, 01/01/1900 als geboortedatum. Rest nog: dit ook in het datamanagementplan zetten.</t>
         </is>
       </c>
       <c r="D40" s="23" t="inlineStr">
@@ -5424,12 +5422,12 @@
       </c>
       <c r="F40" s="23" t="inlineStr">
         <is>
-          <t>Te doen</t>
+          <t>Bezig</t>
         </is>
       </c>
       <c r="G40" s="23" t="inlineStr">
         <is>
-          <t>GDPR</t>
+          <t>Beslist 14 sep; DMP nog</t>
         </is>
       </c>
     </row>
@@ -5475,7 +5473,7 @@
       </c>
       <c r="C42" s="23" t="inlineStr">
         <is>
-          <t>Novel studio bewaart lokaal in C:\Users\Public\Documents\Novel Studio\plidar_data. Vastleggen hoe die bestanden bij het studieteam raken en onder welke naam ze in de database gaan.</t>
+          <t>Deels: de route van de Pressure Monitoring Tool ligt vast (opslaan, mailen naar janou.debuyser@kuleuven.be, lokaal laten staan). Nog open: hoe het geexporteerde pedar-bestand zelf bij het studieteam raakt, en onder welke naam.</t>
         </is>
       </c>
       <c r="D42" s="23" t="inlineStr">
@@ -5490,12 +5488,12 @@
       </c>
       <c r="F42" s="23" t="inlineStr">
         <is>
-          <t>Te doen</t>
+          <t>Bezig</t>
         </is>
       </c>
       <c r="G42" s="23" t="inlineStr">
         <is>
-          <t>Hangt aan de formulierenroute</t>
+          <t>Deels beslist 14 sep</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WP1-afvinklijst: 25% per sessie, tot drie aanpassingen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PARADISE_WP1_afvinklijst.xlsx
+++ b/PARADISE_WP1_afvinklijst.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kuleuven-my.sharepoint.com/personal/janou_debuyser_kuleuven_be1/Documents/Documents/PhD Brugge/Site/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_BD600FB87C3722EDD7AEB33573C921E60A419D9F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1C99987-CE0B-420D-A46A-FA8DD4A5D6B8}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_BD600FB87C3722EDD7AEB33573C921E60A419D9F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55FD3096-EDF3-474D-A7E7-6F8E15AADC44}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overzicht" sheetId="1" r:id="rId1"/>
@@ -1813,16 +1813,16 @@
     <t>Novel Pedar, database en software aanwezig</t>
   </si>
   <si>
-    <t>Pedar als klinisch toestel met trublu-kalibratie; F-Scan GO alleen studieteam; acht regio's; alles in-shoe, zónder én mét de zool gemeten; norm &lt; 200 kPa mét de zool óf ≥ 25% lager dan zonder de zool op visite 2 (vaste referentie, ook op maand 6, 12 en 18); behaalde reductie als fidelity-maat</t>
-  </si>
-  <si>
-    <t>Alles in-shoe, twee condities: zónder en mét de CMFO. De 25%-reductie rekent tegenover de meting zonder zool op visite 2, die ook op maand 6, 12 en 18 de referentie blijft (gepreciseerd op 22 september). Tabel 4 van het manuscript had het goed</t>
-  </si>
-  <si>
     <t>Gedaan, en het bleek meer dan dat: de methodesectie noemde het ontlastingscriterium helemaal niet - 200 kPa en de 25% stonden alleen in de inleiding als beschrijving van de literatuur. Nu staan in de methodesectie de drie doelregio's (vorige ulcusplaats plus de twee voorvoet- of middenvoetregio's boven 200 kPa, hiel niet), de norm met de vergelijking met de meting zonder zool op visite 2 (op 25 september ook zo in het manuscript gezet), en de 5%-stijgingsregel bij opvolging.</t>
   </si>
   <si>
     <t>Gevonden bij het invoegen van het ontlastingscriterium: de sectie Tailoring and fidelity zei dat het ontlastingsdoel tegen de eigen baselinedruk ligt. Rechtgezet naar de meting zonder de zool, conform de beslissing van 11 september; op 22 september gepreciseerd tot de meting zonder zool op visite 2.</t>
+  </si>
+  <si>
+    <t>Pedar als klinisch toestel met trublu-kalibratie; F-Scan GO alleen studieteam; acht regio's; alles in-shoe, zónder én mét de zool gemeten; norm &lt; 200 kPa mét de zool óf ≥ 25% lager dan zonder de zool in dezelfde sessie, tot drie aanpassingen; behaalde reductie als fidelity-maat</t>
+  </si>
+  <si>
+    <t>Alles in-shoe, twee condities: zónder en mét de CMFO. De 25%-reductie rekent tegenover de meting zonder zool in dezelfde sessie, tot drie aanpassingen (beslissing 6 oktober; de vaste referentie van 22 september vervalt). Tabel 4 van het manuscript had het goed</t>
   </si>
 </sst>
 </file>
@@ -2537,7 +2537,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="5" width="10" customWidth="1"/>
@@ -2546,15 +2546,15 @@
     <col min="8" max="8" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="22"/>
       <c r="B4" s="20"/>
       <c r="C4" s="20"/>
@@ -2562,7 +2562,7 @@
       <c r="E4" s="20"/>
       <c r="F4" s="20"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>38</v>
       </c>
@@ -2588,7 +2588,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>45</v>
       </c>
@@ -2621,7 +2621,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>46</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>47</v>
       </c>
@@ -2687,7 +2687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>0</v>
       </c>
@@ -2720,7 +2720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
         <v>48</v>
       </c>
@@ -2753,12 +2753,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
     </row>
   </sheetData>
@@ -2775,7 +2775,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I79"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -2788,7 +2788,7 @@
     <col min="9" max="9" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
         <v>50</v>
       </c>
@@ -2801,7 +2801,7 @@
       <c r="H1" s="20"/>
       <c r="I1" s="20"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
         <v>51</v>
       </c>
@@ -2814,7 +2814,7 @@
       <c r="H2" s="20"/>
       <c r="I2" s="20"/>
     </row>
-    <row r="4" spans="1:9" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>52</v>
       </c>
@@ -2843,7 +2843,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="23" t="s">
         <v>59</v>
       </c>
@@ -2856,7 +2856,7 @@
       <c r="H5" s="24"/>
       <c r="I5" s="25"/>
     </row>
-    <row r="6" spans="1:9" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
         <v>60</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
         <v>68</v>
       </c>
@@ -2914,7 +2914,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>73</v>
       </c>
@@ -2943,7 +2943,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>78</v>
       </c>
@@ -2970,7 +2970,7 @@
       </c>
       <c r="I9" s="10"/>
     </row>
-    <row r="10" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
         <v>83</v>
       </c>
@@ -2999,7 +2999,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>88</v>
       </c>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="I11" s="10"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>94</v>
       </c>
@@ -3053,7 +3053,7 @@
       </c>
       <c r="I12" s="10"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>98</v>
       </c>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="I13" s="10"/>
     </row>
-    <row r="14" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
         <v>102</v>
       </c>
@@ -3109,7 +3109,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
         <v>108</v>
       </c>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="I15" s="10"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="9" t="s">
         <v>114</v>
       </c>
@@ -3165,7 +3165,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" s="23" t="s">
         <v>118</v>
       </c>
@@ -3178,7 +3178,7 @@
       <c r="H17" s="24"/>
       <c r="I17" s="25"/>
     </row>
-    <row r="18" spans="1:9" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="s">
         <v>119</v>
       </c>
@@ -3207,7 +3207,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="9" t="s">
         <v>124</v>
       </c>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="I19" s="10"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" s="9" t="s">
         <v>130</v>
       </c>
@@ -3263,7 +3263,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" s="9" t="s">
         <v>134</v>
       </c>
@@ -3290,7 +3290,7 @@
       </c>
       <c r="I21" s="10"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" s="9" t="s">
         <v>137</v>
       </c>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="I22" s="10"/>
     </row>
-    <row r="23" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="9" t="s">
         <v>140</v>
       </c>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="I23" s="10"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" s="9" t="s">
         <v>143</v>
       </c>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="I24" s="10"/>
     </row>
-    <row r="25" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="9" t="s">
         <v>149</v>
       </c>
@@ -3400,7 +3400,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" s="23" t="s">
         <v>154</v>
       </c>
@@ -3413,7 +3413,7 @@
       <c r="H26" s="24"/>
       <c r="I26" s="25"/>
     </row>
-    <row r="27" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="9" t="s">
         <v>155</v>
       </c>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="I27" s="10"/>
     </row>
-    <row r="28" spans="1:9" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="9" t="s">
         <v>160</v>
       </c>
@@ -3448,7 +3448,7 @@
         <v>161</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D28" s="10" t="s">
         <v>111</v>
@@ -3469,7 +3469,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="9" t="s">
         <v>164</v>
       </c>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="I29" s="10"/>
     </row>
-    <row r="30" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="9" t="s">
         <v>168</v>
       </c>
@@ -3523,7 +3523,7 @@
       </c>
       <c r="I30" s="10"/>
     </row>
-    <row r="31" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="9" t="s">
         <v>174</v>
       </c>
@@ -3550,7 +3550,7 @@
       </c>
       <c r="I31" s="10"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" s="9" t="s">
         <v>178</v>
       </c>
@@ -3577,7 +3577,7 @@
       </c>
       <c r="I32" s="10"/>
     </row>
-    <row r="33" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="9" t="s">
         <v>183</v>
       </c>
@@ -3606,7 +3606,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="9" t="s">
         <v>188</v>
       </c>
@@ -3633,7 +3633,7 @@
       </c>
       <c r="I34" s="10"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" s="23" t="s">
         <v>193</v>
       </c>
@@ -3646,7 +3646,7 @@
       <c r="H35" s="24"/>
       <c r="I35" s="25"/>
     </row>
-    <row r="36" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="9" t="s">
         <v>194</v>
       </c>
@@ -3673,7 +3673,7 @@
       </c>
       <c r="I36" s="10"/>
     </row>
-    <row r="37" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="9" t="s">
         <v>198</v>
       </c>
@@ -3702,7 +3702,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="9" t="s">
         <v>202</v>
       </c>
@@ -3731,7 +3731,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="9" t="s">
         <v>207</v>
       </c>
@@ -3760,7 +3760,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="9" t="s">
         <v>212</v>
       </c>
@@ -3787,7 +3787,7 @@
       </c>
       <c r="I40" s="10"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" s="23" t="s">
         <v>215</v>
       </c>
@@ -3800,7 +3800,7 @@
       <c r="H41" s="24"/>
       <c r="I41" s="25"/>
     </row>
-    <row r="42" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="9" t="s">
         <v>216</v>
       </c>
@@ -3829,7 +3829,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="9" t="s">
         <v>222</v>
       </c>
@@ -3858,7 +3858,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="9" t="s">
         <v>226</v>
       </c>
@@ -3887,7 +3887,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="9" t="s">
         <v>230</v>
       </c>
@@ -3914,7 +3914,7 @@
       </c>
       <c r="I45" s="10"/>
     </row>
-    <row r="46" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="9" t="s">
         <v>235</v>
       </c>
@@ -3943,7 +3943,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" s="9" t="s">
         <v>241</v>
       </c>
@@ -3970,7 +3970,7 @@
       </c>
       <c r="I47" s="10"/>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" s="9" t="s">
         <v>244</v>
       </c>
@@ -3997,7 +3997,7 @@
       </c>
       <c r="I48" s="10"/>
     </row>
-    <row r="49" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="s">
         <v>247</v>
       </c>
@@ -4024,7 +4024,7 @@
       </c>
       <c r="I49" s="10"/>
     </row>
-    <row r="50" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="9" t="s">
         <v>250</v>
       </c>
@@ -4053,7 +4053,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" s="9" t="s">
         <v>255</v>
       </c>
@@ -4082,7 +4082,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="9" t="s">
         <v>260</v>
       </c>
@@ -4111,7 +4111,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" s="23" t="s">
         <v>266</v>
       </c>
@@ -4124,7 +4124,7 @@
       <c r="H53" s="24"/>
       <c r="I53" s="25"/>
     </row>
-    <row r="54" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="9" t="s">
         <v>267</v>
       </c>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="I54" s="10"/>
     </row>
-    <row r="55" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="9" t="s">
         <v>272</v>
       </c>
@@ -4178,7 +4178,7 @@
       </c>
       <c r="I55" s="10"/>
     </row>
-    <row r="56" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="9" t="s">
         <v>275</v>
       </c>
@@ -4207,7 +4207,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="9" t="s">
         <v>282</v>
       </c>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="I57" s="10"/>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" s="9" t="s">
         <v>287</v>
       </c>
@@ -4261,7 +4261,7 @@
       </c>
       <c r="I58" s="10"/>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A59" s="9" t="s">
         <v>290</v>
       </c>
@@ -4290,7 +4290,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A60" s="23" t="s">
         <v>295</v>
       </c>
@@ -4303,7 +4303,7 @@
       <c r="H60" s="24"/>
       <c r="I60" s="25"/>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A61" s="9" t="s">
         <v>296</v>
       </c>
@@ -4330,7 +4330,7 @@
       </c>
       <c r="I61" s="10"/>
     </row>
-    <row r="62" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="9" t="s">
         <v>300</v>
       </c>
@@ -4357,7 +4357,7 @@
       </c>
       <c r="I62" s="10"/>
     </row>
-    <row r="63" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="9" t="s">
         <v>305</v>
       </c>
@@ -4384,7 +4384,7 @@
       </c>
       <c r="I63" s="10"/>
     </row>
-    <row r="64" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="9" t="s">
         <v>308</v>
       </c>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="I64" s="10"/>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" s="23" t="s">
         <v>311</v>
       </c>
@@ -4424,7 +4424,7 @@
       <c r="H65" s="24"/>
       <c r="I65" s="25"/>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" s="9" t="s">
         <v>312</v>
       </c>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="I66" s="10"/>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" s="9" t="s">
         <v>319</v>
       </c>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="I67" s="10"/>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A68" s="9" t="s">
         <v>323</v>
       </c>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="I68" s="10"/>
     </row>
-    <row r="69" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="9" t="s">
         <v>327</v>
       </c>
@@ -4532,7 +4532,7 @@
       </c>
       <c r="I69" s="10"/>
     </row>
-    <row r="70" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="9" t="s">
         <v>330</v>
       </c>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="I70" s="10"/>
     </row>
-    <row r="71" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="9" t="s">
         <v>333</v>
       </c>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="I71" s="10"/>
     </row>
-    <row r="72" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="9" t="s">
         <v>337</v>
       </c>
@@ -4613,7 +4613,7 @@
       </c>
       <c r="I72" s="10"/>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A73" s="23" t="s">
         <v>341</v>
       </c>
@@ -4626,7 +4626,7 @@
       <c r="H73" s="24"/>
       <c r="I73" s="25"/>
     </row>
-    <row r="74" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="9" t="s">
         <v>342</v>
       </c>
@@ -4655,7 +4655,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A75" s="9" t="s">
         <v>347</v>
       </c>
@@ -4682,7 +4682,7 @@
       </c>
       <c r="I75" s="10"/>
     </row>
-    <row r="76" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="9" t="s">
         <v>353</v>
       </c>
@@ -4709,7 +4709,7 @@
       </c>
       <c r="I76" s="10"/>
     </row>
-    <row r="77" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="9" t="s">
         <v>359</v>
       </c>
@@ -4736,7 +4736,7 @@
       </c>
       <c r="I77" s="10"/>
     </row>
-    <row r="78" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="9" t="s">
         <v>362</v>
       </c>
@@ -4763,7 +4763,7 @@
       </c>
       <c r="I78" s="10"/>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A79" s="9" t="s">
         <v>367</v>
       </c>
@@ -4793,17 +4793,17 @@
   </sheetData>
   <autoFilter ref="A4:I79" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="11">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A53:I53"/>
-    <mergeCell ref="A35:I35"/>
-    <mergeCell ref="A26:I26"/>
     <mergeCell ref="A65:I65"/>
     <mergeCell ref="A73:I73"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A41:I41"/>
     <mergeCell ref="A5:I5"/>
     <mergeCell ref="A60:I60"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A53:I53"/>
+    <mergeCell ref="A35:I35"/>
+    <mergeCell ref="A26:I26"/>
   </mergeCells>
   <conditionalFormatting sqref="H5:H79">
     <cfRule type="cellIs" dxfId="17" priority="1" operator="equal">
@@ -4838,7 +4838,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G59"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -4849,7 +4849,7 @@
     <col min="7" max="7" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
         <v>46</v>
       </c>
@@ -4860,7 +4860,7 @@
       <c r="F1" s="20"/>
       <c r="G1" s="20"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
         <v>372</v>
       </c>
@@ -4871,7 +4871,7 @@
       <c r="F2" s="20"/>
       <c r="G2" s="20"/>
     </row>
-    <row r="4" spans="1:7" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>52</v>
       </c>
@@ -4894,7 +4894,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="23" t="s">
         <v>376</v>
       </c>
@@ -4905,7 +4905,7 @@
       <c r="F5" s="24"/>
       <c r="G5" s="25"/>
     </row>
-    <row r="6" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9">
         <v>1</v>
       </c>
@@ -4928,7 +4928,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9">
         <v>2</v>
       </c>
@@ -4951,7 +4951,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9">
         <v>3</v>
       </c>
@@ -4974,7 +4974,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9">
         <v>4</v>
       </c>
@@ -4997,7 +4997,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9">
         <v>5</v>
       </c>
@@ -5020,7 +5020,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9">
         <v>6</v>
       </c>
@@ -5043,7 +5043,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="23" t="s">
         <v>397</v>
       </c>
@@ -5054,7 +5054,7 @@
       <c r="F12" s="24"/>
       <c r="G12" s="25"/>
     </row>
-    <row r="13" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9">
         <v>7</v>
       </c>
@@ -5075,7 +5075,7 @@
       </c>
       <c r="G13" s="10"/>
     </row>
-    <row r="14" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="16">
         <v>8</v>
       </c>
@@ -5098,7 +5098,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="9">
         <v>9</v>
       </c>
@@ -5119,7 +5119,7 @@
       </c>
       <c r="G15" s="10"/>
     </row>
-    <row r="16" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="9">
         <v>10</v>
       </c>
@@ -5142,7 +5142,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="9">
         <v>11</v>
       </c>
@@ -5163,7 +5163,7 @@
       </c>
       <c r="G17" s="10"/>
     </row>
-    <row r="18" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="9">
         <v>12</v>
       </c>
@@ -5186,7 +5186,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="9">
         <v>13</v>
       </c>
@@ -5197,7 +5197,7 @@
       <c r="F19" s="14"/>
       <c r="G19" s="15"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="9">
         <v>14</v>
       </c>
@@ -5220,7 +5220,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A21" s="9">
         <v>15</v>
       </c>
@@ -5243,7 +5243,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="9">
         <v>16</v>
       </c>
@@ -5266,7 +5266,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="23" t="s">
         <v>425</v>
       </c>
@@ -5277,7 +5277,7 @@
       <c r="F23" s="24"/>
       <c r="G23" s="25"/>
     </row>
-    <row r="24" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="9">
         <v>17</v>
       </c>
@@ -5300,7 +5300,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="9">
         <v>18</v>
       </c>
@@ -5323,18 +5323,18 @@
         <v>431</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="18" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A28" s="16"/>
       <c r="B28" s="17" t="s">
         <v>433</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="D28" s="17" t="s">
         <v>434</v>
@@ -5349,7 +5349,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="52" x14ac:dyDescent="0.35">
       <c r="A29" s="16"/>
       <c r="B29" s="17" t="s">
         <v>436</v>
@@ -5370,7 +5370,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A30" s="16"/>
       <c r="B30" s="17" t="s">
         <v>439</v>
@@ -5391,7 +5391,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="26" x14ac:dyDescent="0.35">
       <c r="A31" s="16"/>
       <c r="B31" s="17" t="s">
         <v>443</v>
@@ -5412,7 +5412,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="26" x14ac:dyDescent="0.35">
       <c r="A32" s="16"/>
       <c r="B32" s="17" t="s">
         <v>447</v>
@@ -5433,7 +5433,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="26" x14ac:dyDescent="0.35">
       <c r="A33" s="16"/>
       <c r="B33" s="17" t="s">
         <v>451</v>
@@ -5454,7 +5454,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" ht="26" x14ac:dyDescent="0.35">
       <c r="A34" s="16"/>
       <c r="B34" s="17" t="s">
         <v>455</v>
@@ -5475,7 +5475,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A35" s="16"/>
       <c r="B35" s="17" t="s">
         <v>458</v>
@@ -5496,7 +5496,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" ht="26" x14ac:dyDescent="0.35">
       <c r="A36" s="16"/>
       <c r="B36" s="17" t="s">
         <v>461</v>
@@ -5517,7 +5517,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" ht="26" x14ac:dyDescent="0.35">
       <c r="A37" s="16"/>
       <c r="B37" s="17" t="s">
         <v>464</v>
@@ -5538,7 +5538,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A38" s="16"/>
       <c r="B38" s="17" t="s">
         <v>468</v>
@@ -5559,7 +5559,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" ht="52" x14ac:dyDescent="0.35">
       <c r="A39" s="16"/>
       <c r="B39" s="17" t="s">
         <v>472</v>
@@ -5580,7 +5580,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="26" x14ac:dyDescent="0.35">
       <c r="A40" s="16"/>
       <c r="B40" s="17" t="s">
         <v>475</v>
@@ -5601,7 +5601,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A41" s="16"/>
       <c r="B41" s="17" t="s">
         <v>479</v>
@@ -5622,7 +5622,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A42" s="16"/>
       <c r="B42" s="17" t="s">
         <v>482</v>
@@ -5643,7 +5643,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A43" s="16"/>
       <c r="B43" s="17" t="s">
         <v>486</v>
@@ -5664,7 +5664,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" ht="26" x14ac:dyDescent="0.35">
       <c r="A44" s="16"/>
       <c r="B44" s="17" t="s">
         <v>489</v>
@@ -5685,7 +5685,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="26" x14ac:dyDescent="0.35">
       <c r="A45" s="16"/>
       <c r="B45" s="17" t="s">
         <v>491</v>
@@ -5706,7 +5706,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A46" s="16"/>
       <c r="B46" s="17" t="s">
         <v>494</v>
@@ -5727,7 +5727,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A47" s="16"/>
       <c r="B47" s="17" t="s">
         <v>497</v>
@@ -5748,7 +5748,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="26" x14ac:dyDescent="0.35">
       <c r="A48" s="16"/>
       <c r="B48" s="17" t="s">
         <v>499</v>
@@ -5769,7 +5769,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A49" s="16"/>
       <c r="B49" s="17" t="s">
         <v>503</v>
@@ -5790,7 +5790,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" ht="26" x14ac:dyDescent="0.35">
       <c r="A50" s="16"/>
       <c r="B50" s="17" t="s">
         <v>506</v>
@@ -5811,7 +5811,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A51" s="16"/>
       <c r="B51" s="17" t="s">
         <v>508</v>
@@ -5832,7 +5832,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="16"/>
       <c r="B52" s="17" t="s">
         <v>511</v>
@@ -5853,7 +5853,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="78" x14ac:dyDescent="0.35">
       <c r="A53" s="16"/>
       <c r="B53" s="17" t="s">
         <v>514</v>
@@ -5874,13 +5874,13 @@
         <v>517</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="78" x14ac:dyDescent="0.35">
       <c r="A54" s="16"/>
       <c r="B54" s="17" t="s">
         <v>518</v>
       </c>
       <c r="C54" s="17" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="D54" s="17" t="s">
         <v>519</v>
@@ -5895,7 +5895,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A55" s="16"/>
       <c r="B55" s="17" t="s">
         <v>520</v>
@@ -5916,7 +5916,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="16"/>
       <c r="B56" s="17" t="s">
         <v>522</v>
@@ -5937,7 +5937,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" ht="52" x14ac:dyDescent="0.35">
       <c r="A57" s="16"/>
       <c r="B57" s="17" t="s">
         <v>524</v>
@@ -5958,7 +5958,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="58" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" ht="39" x14ac:dyDescent="0.35">
       <c r="A58" s="16"/>
       <c r="B58" s="17" t="s">
         <v>526</v>
@@ -5979,13 +5979,13 @@
         <v>529</v>
       </c>
     </row>
-    <row r="59" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" ht="52" x14ac:dyDescent="0.35">
       <c r="A59" s="16"/>
       <c r="B59" s="17" t="s">
         <v>530</v>
       </c>
       <c r="C59" s="17" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="D59" s="17" t="s">
         <v>531</v>
@@ -6039,7 +6039,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="52" customWidth="1"/>
@@ -6051,7 +6051,7 @@
     <col min="11" max="11" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
         <v>533</v>
       </c>
@@ -6061,7 +6061,7 @@
       <c r="E1" s="20"/>
       <c r="F1" s="20"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
         <v>534</v>
       </c>
@@ -6071,7 +6071,7 @@
       <c r="E2" s="20"/>
       <c r="F2" s="20"/>
     </row>
-    <row r="4" spans="1:11" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>52</v>
       </c>
@@ -6091,7 +6091,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="23" t="s">
         <v>538</v>
       </c>
@@ -6101,7 +6101,7 @@
       <c r="E5" s="24"/>
       <c r="F5" s="25"/>
     </row>
-    <row r="6" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9">
         <v>1</v>
       </c>
@@ -6119,7 +6119,7 @@
       </c>
       <c r="F6" s="10"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="9">
         <v>2</v>
       </c>
@@ -6139,7 +6139,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="9">
         <v>3</v>
       </c>
@@ -6157,7 +6157,7 @@
       </c>
       <c r="F8" s="10"/>
     </row>
-    <row r="9" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9">
         <v>4</v>
       </c>
@@ -6175,7 +6175,7 @@
       </c>
       <c r="F9" s="10"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" s="9">
         <v>5</v>
       </c>
@@ -6193,7 +6193,7 @@
       </c>
       <c r="F10" s="10"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="9">
         <v>6</v>
       </c>
@@ -6213,7 +6213,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9">
         <v>7</v>
       </c>
@@ -6233,12 +6233,12 @@
         <v>561</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="11" t="s">
         <v>562</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
         <v>52</v>
       </c>
@@ -6273,7 +6273,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" s="9">
         <v>1</v>
       </c>
@@ -6294,7 +6294,7 @@
       </c>
       <c r="K16" s="9"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="9">
         <v>2</v>
       </c>
@@ -6315,7 +6315,7 @@
       </c>
       <c r="K17" s="9"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="9">
         <v>3</v>
       </c>
@@ -6336,7 +6336,7 @@
       </c>
       <c r="K18" s="9"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="9">
         <v>4</v>
       </c>
@@ -6357,7 +6357,7 @@
       </c>
       <c r="K19" s="9"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" s="9">
         <v>5</v>
       </c>
@@ -6378,7 +6378,7 @@
       </c>
       <c r="K20" s="9"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" s="9">
         <v>6</v>
       </c>
@@ -6399,7 +6399,7 @@
       </c>
       <c r="K21" s="9"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" s="9">
         <v>7</v>
       </c>
@@ -6420,7 +6420,7 @@
       </c>
       <c r="K22" s="9"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="9">
         <v>8</v>
       </c>
@@ -6441,7 +6441,7 @@
       </c>
       <c r="K23" s="9"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" s="9">
         <v>9</v>
       </c>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="K24" s="9"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="12">
         <v>10</v>
       </c>
@@ -6527,7 +6527,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
     <col min="2" max="2" width="46" customWidth="1"/>
@@ -6537,7 +6537,7 @@
     <col min="7" max="7" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -6548,7 +6548,7 @@
       <c r="F1" s="20"/>
       <c r="G1" s="20"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
         <v>1</v>
       </c>
@@ -6559,7 +6559,7 @@
       <c r="F2" s="20"/>
       <c r="G2" s="20"/>
     </row>
-    <row r="4" spans="1:7" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
@@ -6582,7 +6582,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
         <v>9</v>
       </c>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="G5" s="10"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
         <v>15</v>
       </c>
@@ -6624,7 +6624,7 @@
       </c>
       <c r="G6" s="10"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
         <v>18</v>
       </c>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="G7" s="10"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>21</v>
       </c>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="G8" s="10"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>26</v>
       </c>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="G9" s="10"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
         <v>31</v>
       </c>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="G10" s="10"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>33</v>
       </c>

</xml_diff>